<commit_message>
Update 1 Januari 2020
</commit_message>
<xml_diff>
--- a/Projects/RAB.xlsx
+++ b/Projects/RAB.xlsx
@@ -7,8 +7,8 @@
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="RAB" sheetId="1" r:id="rId1"/>
+    <sheet name="Plan" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="125725"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>No</t>
   </si>
@@ -61,6 +61,39 @@
   </si>
   <si>
     <t>GPS</t>
+  </si>
+  <si>
+    <t>Power</t>
+  </si>
+  <si>
+    <t>5v</t>
+  </si>
+  <si>
+    <t>3.7v</t>
+  </si>
+  <si>
+    <t>Ublox Neo 6m</t>
+  </si>
+  <si>
+    <t>Batrai</t>
+  </si>
+  <si>
+    <t>Li-Ion 18650</t>
+  </si>
+  <si>
+    <t>Micro Usb</t>
+  </si>
+  <si>
+    <t>Solid State Ralay</t>
+  </si>
+  <si>
+    <t>Step Down</t>
+  </si>
+  <si>
+    <t>Charger Li-Ion</t>
+  </si>
+  <si>
+    <t>HT7333-A</t>
   </si>
 </sst>
 </file>
@@ -396,8 +429,8 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="3.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7.28515625" bestFit="1" customWidth="1"/>
@@ -471,30 +504,54 @@
       <c r="C6" t="s">
         <v>14</v>
       </c>
+      <c r="D6" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="7" spans="2:9">
       <c r="B7">
         <v>5</v>
       </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="8" spans="2:9">
       <c r="B8">
         <v>6</v>
       </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="9" spans="2:9">
       <c r="B9">
         <v>7</v>
       </c>
+      <c r="C9" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="10" spans="2:9">
       <c r="B10">
         <v>8</v>
       </c>
+      <c r="C10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="11" spans="2:9">
       <c r="B11">
         <v>9</v>
+      </c>
+      <c r="C11" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="2:9">
@@ -609,9 +666,28 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="6.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Make Folder Project ESP32
</commit_message>
<xml_diff>
--- a/Projects/RAB.xlsx
+++ b/Projects/RAB.xlsx
@@ -9,14 +9,14 @@
   <sheets>
     <sheet name="RAB" sheetId="1" r:id="rId1"/>
     <sheet name="Plan" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="BlockDiaram" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="35">
   <si>
     <t>No</t>
   </si>
@@ -94,6 +94,33 @@
   </si>
   <si>
     <t>HT7333-A</t>
+  </si>
+  <si>
+    <t>USB</t>
+  </si>
+  <si>
+    <t>Charger</t>
+  </si>
+  <si>
+    <t>MU</t>
+  </si>
+  <si>
+    <t>A6</t>
+  </si>
+  <si>
+    <t>Remote RF</t>
+  </si>
+  <si>
+    <t>mongcicit</t>
+  </si>
+  <si>
+    <t>Batrai Holder</t>
+  </si>
+  <si>
+    <t>LDO</t>
+  </si>
+  <si>
+    <t>Switch on/off</t>
   </si>
 </sst>
 </file>
@@ -109,12 +136,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -129,8 +162,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -474,6 +511,7 @@
       <c r="D3" t="s">
         <v>8</v>
       </c>
+      <c r="I3" s="1"/>
     </row>
     <row r="4" spans="2:9">
       <c r="B4">
@@ -485,6 +523,7 @@
       <c r="D4" t="s">
         <v>9</v>
       </c>
+      <c r="I4" s="1"/>
     </row>
     <row r="5" spans="2:9">
       <c r="B5">
@@ -496,6 +535,9 @@
       <c r="D5" t="s">
         <v>13</v>
       </c>
+      <c r="I5" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="6" spans="2:9">
       <c r="B6">
@@ -507,6 +549,7 @@
       <c r="D6" t="s">
         <v>18</v>
       </c>
+      <c r="I6" s="1"/>
     </row>
     <row r="7" spans="2:9">
       <c r="B7">
@@ -518,6 +561,7 @@
       <c r="D7" t="s">
         <v>20</v>
       </c>
+      <c r="I7" s="1"/>
     </row>
     <row r="8" spans="2:9">
       <c r="B8">
@@ -526,6 +570,7 @@
       <c r="C8" t="s">
         <v>21</v>
       </c>
+      <c r="I8" s="1"/>
     </row>
     <row r="9" spans="2:9">
       <c r="B9">
@@ -553,20 +598,32 @@
       <c r="C11" t="s">
         <v>24</v>
       </c>
+      <c r="I11" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="12" spans="2:9">
       <c r="B12">
         <v>10</v>
       </c>
+      <c r="C12" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="13" spans="2:9">
       <c r="B13">
         <v>11</v>
       </c>
+      <c r="C13" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="14" spans="2:9">
       <c r="B14">
         <v>12</v>
+      </c>
+      <c r="C14" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="2:9">
@@ -694,9 +751,47 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="B4:F6"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="4.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="2:6">
+      <c r="D4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6">
+      <c r="B5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6">
+      <c r="E6" s="2"/>
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="E5:E6"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>